<commit_message>
ระบบ import template user ได้ละ
</commit_message>
<xml_diff>
--- a/public/templates/User_Template.xlsx
+++ b/public/templates/User_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\competency-v1\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA66E7F9-6C83-4066-8392-AE4A0572EDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9001EA-4CD8-4BA9-A561-7A944803417F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="117">
   <si>
     <t>📋  User Import Template — ระบบ Competency &amp; IDP คณะวิศวกรรมศาสตร์ มข.</t>
   </si>
@@ -86,9 +86,6 @@
     <t>สายงาน *</t>
   </si>
   <si>
-    <t>กลุ่มงาน (Division) *</t>
-  </si>
-  <si>
     <t>ตำแหน่ง *</t>
   </si>
   <si>
@@ -116,12 +113,6 @@
     <t>สนับสนุน</t>
   </si>
   <si>
-    <t>งานแผนยุทธศาสตร์ฯ</t>
-  </si>
-  <si>
-    <t>นักวิชาการคอมพิวเตอร์</t>
-  </si>
-  <si>
     <t>ชำนาญการ</t>
   </si>
   <si>
@@ -354,6 +345,33 @@
   </si>
   <si>
     <t>user</t>
+  </si>
+  <si>
+    <t>ฝ่าย</t>
+  </si>
+  <si>
+    <t>งาน</t>
+  </si>
+  <si>
+    <t>แผนยุทธศาสตร์และทรัพยากรบุคคล</t>
+  </si>
+  <si>
+    <t>แผนยุทธศาสตร์และพัฒนาองค์กร</t>
+  </si>
+  <si>
+    <t>job</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บริหารการเงินและพัสดุ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">นักวิชาการเงินและบัญชี </t>
+  </si>
+  <si>
+    <t>กลุ่มงาน*</t>
+  </si>
+  <si>
+    <t>job_family</t>
   </si>
 </sst>
 </file>
@@ -679,6 +697,12 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -690,12 +714,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -999,7 +1017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1009,44 +1027,50 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="9" width="22" customWidth="1"/>
-    <col min="10" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="22" style="21" customWidth="1"/>
+    <col min="8" max="8" width="23.69921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="22" customWidth="1"/>
+    <col min="12" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="22" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="22"/>
-    </row>
-    <row r="2" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="22"/>
+    </row>
+    <row r="2" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="23"/>
-    </row>
-    <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="23"/>
+    </row>
+    <row r="3" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1072,17 +1096,23 @@
         <v>9</v>
       </c>
       <c r="I3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="19"/>
-    </row>
-    <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="19"/>
+    </row>
+    <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1105,56 +1135,68 @@
         <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="M4" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="N4" s="25"/>
+    </row>
+    <row r="5" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="L4" s="25"/>
-    </row>
-    <row r="5" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="L5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="L5" s="24"/>
-    </row>
-    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M5" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="N5" s="24"/>
+    </row>
+    <row r="6" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1166,9 +1208,11 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="20"/>
-    </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="20"/>
+    </row>
+    <row r="7" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1180,9 +1224,11 @@
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
-      <c r="L7" s="20"/>
-    </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="20"/>
+    </row>
+    <row r="8" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1194,9 +1240,11 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
-      <c r="L8" s="20"/>
-    </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="20"/>
+    </row>
+    <row r="9" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1208,9 +1256,11 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
-      <c r="L9" s="20"/>
-    </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="20"/>
+    </row>
+    <row r="10" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1222,9 +1272,11 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
-      <c r="L10" s="20"/>
-    </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="20"/>
+    </row>
+    <row r="11" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1236,9 +1288,11 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="L11" s="20"/>
-    </row>
-    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="20"/>
+    </row>
+    <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1250,9 +1304,11 @@
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
-      <c r="L12" s="20"/>
-    </row>
-    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="20"/>
+    </row>
+    <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1264,9 +1320,11 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
-      <c r="L13" s="20"/>
-    </row>
-    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="20"/>
+    </row>
+    <row r="14" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1278,9 +1336,11 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
-      <c r="L14" s="20"/>
-    </row>
-    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="20"/>
+    </row>
+    <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1292,9 +1352,11 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
-      <c r="L15" s="20"/>
-    </row>
-    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="20"/>
+    </row>
+    <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1306,9 +1368,11 @@
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
-      <c r="L16" s="20"/>
-    </row>
-    <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="20"/>
+    </row>
+    <row r="17" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1320,9 +1384,11 @@
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
-      <c r="L17" s="20"/>
-    </row>
-    <row r="18" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="20"/>
+    </row>
+    <row r="18" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1334,9 +1400,11 @@
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
-      <c r="L18" s="20"/>
-    </row>
-    <row r="19" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="20"/>
+    </row>
+    <row r="19" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1348,9 +1416,11 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
-      <c r="L19" s="20"/>
-    </row>
-    <row r="20" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="20"/>
+    </row>
+    <row r="20" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1362,9 +1432,11 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
-      <c r="L20" s="20"/>
-    </row>
-    <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="20"/>
+    </row>
+    <row r="21" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1376,9 +1448,11 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
-      <c r="L21" s="20"/>
-    </row>
-    <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="20"/>
+    </row>
+    <row r="22" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1390,9 +1464,11 @@
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
-      <c r="L22" s="20"/>
-    </row>
-    <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="20"/>
+    </row>
+    <row r="23" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1404,9 +1480,11 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
-      <c r="L23" s="20"/>
-    </row>
-    <row r="24" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="20"/>
+    </row>
+    <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1418,9 +1496,11 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
-      <c r="L24" s="20"/>
-    </row>
-    <row r="25" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="20"/>
+    </row>
+    <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1432,9 +1512,11 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
-      <c r="L25" s="20"/>
-    </row>
-    <row r="26" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="20"/>
+    </row>
+    <row r="26" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1446,9 +1528,11 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
-      <c r="L26" s="20"/>
-    </row>
-    <row r="27" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="20"/>
+    </row>
+    <row r="27" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1460,9 +1544,11 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
-      <c r="L27" s="20"/>
-    </row>
-    <row r="28" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="20"/>
+    </row>
+    <row r="28" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1474,9 +1560,11 @@
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
-      <c r="L28" s="20"/>
-    </row>
-    <row r="29" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="20"/>
+    </row>
+    <row r="29" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1488,9 +1576,11 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
-      <c r="L29" s="20"/>
-    </row>
-    <row r="30" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="20"/>
+    </row>
+    <row r="30" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -1502,12 +1592,14 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
-      <c r="L30" s="20"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1523,12 +1615,12 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1536,21 +1628,21 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1558,10 +1650,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1569,10 +1661,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1580,10 +1672,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1591,264 +1683,264 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C32" s="13"/>
     </row>
     <row r="33" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C33" s="10"/>
     </row>
     <row r="34" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>98</v>
       </c>
       <c r="C34" s="13"/>
     </row>
     <row r="35" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C35" s="10"/>
     </row>
     <row r="36" spans="1:3" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1856,7 +1948,7 @@
         <v>9</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1864,7 +1956,7 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1872,7 +1964,7 @@
         <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1880,7 +1972,7 @@
         <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>